<commit_message>
Thu Jul 23 00:33:59 EEST 2026
</commit_message>
<xml_diff>
--- a/TLS_Germany/firest is excel and google sheet have same extent.xlsx
+++ b/TLS_Germany/firest is excel and google sheet have same extent.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Account</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>moed-TLS-25</t>
+  </si>
+  <si>
+    <t>tonil42212@rapplo.com</t>
   </si>
 </sst>
 </file>
@@ -477,10 +480,18 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="2"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1">
+        <v>58.0</v>
+      </c>
+      <c r="D4" s="1">
+        <v>200.0</v>
+      </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="1"/>

</xml_diff>

<commit_message>
Tue Jul 28 23:40:39 EEST 2026
</commit_message>
<xml_diff>
--- a/TLS_Germany/firest is excel and google sheet have same extent.xlsx
+++ b/TLS_Germany/firest is excel and google sheet have same extent.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -108,9 +108,6 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -401,7 +398,9 @@
       <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="H2" s="1">
+        <v>2026.0</v>
+      </c>
       <c r="I2" s="4"/>
       <c r="J2" s="1"/>
       <c r="K2" s="2"/>
@@ -439,7 +438,9 @@
       <c r="G3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="5"/>
+      <c r="H3" s="1">
+        <v>2026.0</v>
+      </c>
       <c r="I3" s="4"/>
       <c r="J3" s="1"/>
       <c r="K3" s="2"/>
@@ -477,7 +478,9 @@
       <c r="G4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="1">
+        <v>2026.0</v>
+      </c>
       <c r="I4" s="4"/>
       <c r="J4" s="1"/>
       <c r="K4" s="2"/>

</xml_diff>